<commit_message>
docs(ml): update EDA, SHAP diagrams, and evaluation metrics for corrected pipeline
</commit_message>
<xml_diff>
--- a/training/reports/training_results.xlsx
+++ b/training/reports/training_results.xlsx
@@ -506,56 +506,56 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>LightGBM</t>
         </is>
       </c>
       <c r="B2" t="n">
+        <v>0.99968</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.9996638046963898</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.9999223963991929</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.9997930838269147</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.9999978356016821</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.9999993645260307</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.9993881070340171</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.9990875923306585</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.9990874298258632</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.001337114897458865</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1.724119186401367</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.05129599571228027</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1083.296875</v>
+      </c>
+      <c r="O2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="n">
+      <c r="P2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.002191939782841218</v>
-      </c>
-      <c r="L2" t="n">
-        <v>5.0453200340271</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.02706694602966309</v>
-      </c>
-      <c r="N2" t="n">
-        <v>883.625</v>
-      </c>
-      <c r="O2" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="P2" t="n">
-        <v>2.5</v>
-      </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -565,162 +565,162 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0.99944</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>0.9995861569499768</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0.9996895855967717</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0.9996378685980342</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0.9999926857477286</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>0.9999978524367834</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>0.9991394498253652</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0.998403326684613</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>0.9984033007113678</v>
       </c>
       <c r="K3" t="n">
-        <v>3.763255153899081e-05</v>
+        <v>0.002548699267208576</v>
       </c>
       <c r="L3" t="n">
-        <v>3.331317186355591</v>
+        <v>2.788061857223511</v>
       </c>
       <c r="M3" t="n">
-        <v>0.04286098480224609</v>
+        <v>0.03443002700805664</v>
       </c>
       <c r="N3" t="n">
-        <v>894.5</v>
+        <v>923.75</v>
       </c>
       <c r="O3" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="P3" t="n">
         <v>2.5</v>
       </c>
       <c r="Q3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0.99936</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>0.9994827497025811</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0.9996895855967717</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0.9995861569499768</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0.9999913355645841</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>0.9999974441928484</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>0.99896311408211</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0.9981750772814465</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0.9981749733863213</v>
       </c>
       <c r="K4" t="n">
-        <v>7.867809999058968e-05</v>
+        <v>0.0038413127711533</v>
       </c>
       <c r="L4" t="n">
-        <v>1.067628622055054</v>
+        <v>1.981523036956787</v>
       </c>
       <c r="M4" t="n">
-        <v>0.05940699577331543</v>
+        <v>0.03217911720275879</v>
       </c>
       <c r="N4" t="n">
-        <v>1105.75</v>
+        <v>1117.765625</v>
       </c>
       <c r="O4" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="P4" t="n">
         <v>2.5</v>
       </c>
       <c r="Q4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="B5" t="n">
+        <v>0.9987</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.9992755310616057</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.9990428889233793</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.9991591964505154</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9999862974656543</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.9999959768091486</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.9982870942589035</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.9962950083336186</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.9962948772279411</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.004666646833016646</v>
+      </c>
+      <c r="L5" t="n">
+        <v>13.99202299118042</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.03044462203979492</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1068.359375</v>
+      </c>
+      <c r="O5" t="n">
+        <v>4</v>
+      </c>
+      <c r="P5" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q5" t="n">
         <v>1</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.006065224701658206</v>
-      </c>
-      <c r="L5" t="n">
-        <v>2.739871978759766</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.07170414924621582</v>
-      </c>
-      <c r="N5" t="n">
-        <v>773</v>
-      </c>
-      <c r="O5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="P5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(ml): implement strict leakage-free validation and StratifiedKFold CV
</commit_message>
<xml_diff>
--- a/training/reports/training_results.xlsx
+++ b/training/reports/training_results.xlsx
@@ -506,47 +506,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.99968</v>
+        <v>0.99946</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9996638046963898</v>
+        <v>0.9996378592307096</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9999223963991929</v>
+        <v>0.999663717729836</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9997930838269147</v>
+        <v>0.9996507883130489</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9999978356016821</v>
+        <v>0.999992231885489</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9999993645260307</v>
+        <v>0.9999977153469848</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9993881070340171</v>
+        <v>0.999214683763525</v>
       </c>
       <c r="I2" t="n">
-        <v>0.9990875923306585</v>
+        <v>0.9984604711961367</v>
       </c>
       <c r="J2" t="n">
-        <v>0.9990874298258632</v>
+        <v>0.9984604695730194</v>
       </c>
       <c r="K2" t="n">
-        <v>0.001337114897458865</v>
+        <v>0.002799605823411633</v>
       </c>
       <c r="L2" t="n">
-        <v>1.724119186401367</v>
+        <v>5.849040031433105</v>
       </c>
       <c r="M2" t="n">
-        <v>0.05129599571228027</v>
+        <v>0.02867984771728516</v>
       </c>
       <c r="N2" t="n">
-        <v>1083.296875</v>
+        <v>1140.453125</v>
       </c>
       <c r="O2" t="n">
         <v>1</v>
@@ -555,114 +555,114 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>LightGBM</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.99944</v>
+        <v>0.9993</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9995861569499768</v>
+        <v>0.9995602348863077</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9996895855967717</v>
+        <v>0.9995343783951576</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9996378685980342</v>
+        <v>0.9995473064735174</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9999926857477286</v>
+        <v>0.9999925169748356</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9999978524367834</v>
+        <v>0.9999977967435838</v>
       </c>
       <c r="H3" t="n">
-        <v>0.9991394498253652</v>
+        <v>0.9990177622887444</v>
       </c>
       <c r="I3" t="n">
-        <v>0.998403326684613</v>
+        <v>0.9980044383591169</v>
       </c>
       <c r="J3" t="n">
-        <v>0.9984033007113678</v>
+        <v>0.9980044367369431</v>
       </c>
       <c r="K3" t="n">
-        <v>0.002548699267208576</v>
+        <v>0.002824865275081044</v>
       </c>
       <c r="L3" t="n">
-        <v>2.788061857223511</v>
+        <v>1.202428817749023</v>
       </c>
       <c r="M3" t="n">
-        <v>0.03443002700805664</v>
+        <v>0.06691622734069824</v>
       </c>
       <c r="N3" t="n">
-        <v>923.75</v>
+        <v>917.0625</v>
       </c>
       <c r="O3" t="n">
         <v>2</v>
       </c>
       <c r="P3" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="Q3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.99936</v>
+        <v>0.99918</v>
       </c>
       <c r="C4" t="n">
-        <v>0.9994827497025811</v>
+        <v>0.9993276267811425</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9996895855967717</v>
+        <v>0.9996119819959646</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9995861569499768</v>
+        <v>0.9994697841633582</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9999913355645841</v>
+        <v>0.9999904255593901</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9999974441928484</v>
+        <v>0.9999971854635314</v>
       </c>
       <c r="H4" t="n">
-        <v>0.99896311408211</v>
+        <v>0.9986598086668237</v>
       </c>
       <c r="I4" t="n">
-        <v>0.9981750772814465</v>
+        <v>0.9976616624231431</v>
       </c>
       <c r="J4" t="n">
-        <v>0.9981749733863213</v>
+        <v>0.9976614660607384</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0038413127711533</v>
+        <v>0.01151030231267214</v>
       </c>
       <c r="L4" t="n">
-        <v>1.981523036956787</v>
+        <v>1.837137222290039</v>
       </c>
       <c r="M4" t="n">
-        <v>0.03217911720275879</v>
+        <v>0.03249597549438477</v>
       </c>
       <c r="N4" t="n">
-        <v>1117.765625</v>
+        <v>934.640625</v>
       </c>
       <c r="O4" t="n">
         <v>3</v>
       </c>
       <c r="P4" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="Q4" t="n">
         <v>2</v>
@@ -671,47 +671,47 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9987</v>
+        <v>0.99914</v>
       </c>
       <c r="C5" t="n">
-        <v>0.9992755310616057</v>
+        <v>0.9993792514807439</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9990428889233793</v>
+        <v>0.9995085105282219</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9991591964505154</v>
+        <v>0.9994438768251833</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9999862974656543</v>
+        <v>0.999989599940643</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9999959768091486</v>
+        <v>0.9999969400633786</v>
       </c>
       <c r="H5" t="n">
-        <v>0.9982870942589035</v>
+        <v>0.99869624080458</v>
       </c>
       <c r="I5" t="n">
-        <v>0.9962950083336186</v>
+        <v>0.9975478902494018</v>
       </c>
       <c r="J5" t="n">
-        <v>0.9962948772279411</v>
+        <v>0.9975478496984514</v>
       </c>
       <c r="K5" t="n">
-        <v>0.004666646833016646</v>
+        <v>0.004943434681141869</v>
       </c>
       <c r="L5" t="n">
-        <v>13.99202299118042</v>
+        <v>2.571784973144531</v>
       </c>
       <c r="M5" t="n">
-        <v>0.03044462203979492</v>
+        <v>0.05972719192504883</v>
       </c>
       <c r="N5" t="n">
-        <v>1068.359375</v>
+        <v>1122</v>
       </c>
       <c r="O5" t="n">
         <v>4</v>
@@ -720,7 +720,7 @@
         <v>4</v>
       </c>
       <c r="Q5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(phase2): update Phase 2 data audit reports, figures, and exports
</commit_message>
<xml_diff>
--- a/training/reports/training_results.xlsx
+++ b/training/reports/training_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,47 +506,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.99946</v>
+        <v>0.99964</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9996378592307096</v>
+        <v>0.999637943519189</v>
       </c>
       <c r="D2" t="n">
-        <v>0.999663717729836</v>
+        <v>0.9998965285322572</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9996507883130489</v>
+        <v>0.9997672193052789</v>
       </c>
       <c r="F2" t="n">
-        <v>0.999992231885489</v>
+        <v>0.9999934999629019</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9999977153469848</v>
+        <v>0.9999980857553534</v>
       </c>
       <c r="H2" t="n">
-        <v>0.999214683763525</v>
+        <v>0.9993310891647356</v>
       </c>
       <c r="I2" t="n">
-        <v>0.9984604711961367</v>
+        <v>0.9989735210403372</v>
       </c>
       <c r="J2" t="n">
-        <v>0.9984604695730194</v>
+        <v>0.9989733585540961</v>
       </c>
       <c r="K2" t="n">
-        <v>0.002799605823411633</v>
+        <v>0.002626628119524875</v>
       </c>
       <c r="L2" t="n">
-        <v>5.849040031433105</v>
+        <v>6.762012958526611</v>
       </c>
       <c r="M2" t="n">
-        <v>0.02867984771728516</v>
+        <v>0.09522724151611328</v>
       </c>
       <c r="N2" t="n">
-        <v>1140.453125</v>
+        <v>884.59375</v>
       </c>
       <c r="O2" t="n">
         <v>1</v>
@@ -556,171 +556,6 @@
       </c>
       <c r="Q2" t="n">
         <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>LightGBM</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0.9993</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.9995602348863077</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.9995343783951576</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.9995473064735174</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.9999925169748356</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.9999977967435838</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.9990177622887444</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.9980044383591169</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.9980044367369431</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.002824865275081044</v>
-      </c>
-      <c r="L3" t="n">
-        <v>1.202428817749023</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.06691622734069824</v>
-      </c>
-      <c r="N3" t="n">
-        <v>917.0625</v>
-      </c>
-      <c r="O3" t="n">
-        <v>2</v>
-      </c>
-      <c r="P3" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0.99918</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.9993276267811425</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.9996119819959646</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.9994697841633582</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.9999904255593901</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.9999971854635314</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.9986598086668237</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.9976616624231431</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.9976614660607384</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.01151030231267214</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1.837137222290039</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.03249597549438477</v>
-      </c>
-      <c r="N4" t="n">
-        <v>934.640625</v>
-      </c>
-      <c r="O4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Random Forest</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0.99914</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.9993792514807439</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.9995085105282219</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.9994438768251833</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.999989599940643</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.9999969400633786</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.99869624080458</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.9975478902494018</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.9975478496984514</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.004943434681141869</v>
-      </c>
-      <c r="L5" t="n">
-        <v>2.571784973144531</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.05972719192504883</v>
-      </c>
-      <c r="N5" t="n">
-        <v>1122</v>
-      </c>
-      <c r="O5" t="n">
-        <v>4</v>
-      </c>
-      <c r="P5" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>